<commit_message>
Update Sprint 2 ADAPT_Blueprint
</commit_message>
<xml_diff>
--- a/docs/Sprint-2/Sprint 2 ADAPT_Blueprint.xlsx
+++ b/docs/Sprint-2/Sprint 2 ADAPT_Blueprint.xlsx
@@ -239,9 +239,9 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>-171450</xdr:rowOff>
+      <xdr:rowOff>-180975</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="12773025" cy="13249275"/>
+    <xdr:ext cx="12753975" cy="13192125"/>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
         <xdr:cNvPr id="2" name="Shape 2" title="ภาพวาด"/>
@@ -249,10 +249,10 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="1515700" y="152400"/>
-          <a:ext cx="7638457" cy="7924803"/>
-          <a:chOff x="1515700" y="152400"/>
-          <a:chExt cx="7638457" cy="7924803"/>
+          <a:off x="152400" y="152400"/>
+          <a:ext cx="7653935" cy="7924803"/>
+          <a:chOff x="152400" y="152400"/>
+          <a:chExt cx="7653935" cy="7924803"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:pic>
@@ -270,8 +270,8 @@
         </xdr:blipFill>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="1515700" y="152400"/>
-            <a:ext cx="7638457" cy="7924803"/>
+            <a:off x="152400" y="152400"/>
+            <a:ext cx="7653935" cy="7924803"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>

</xml_diff>